<commit_message>
feat: implement P0 and P1 audit fixes including ettoday registry, MathJax rendering, pollster weight transparency table, weight split display, and 3 new 2026 polls
</commit_message>
<xml_diff>
--- a/sheets_import/clearpoll_database.xlsx
+++ b/sheets_import/clearpoll_database.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -533,51 +533,153 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>nt2026-001b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>zmedia</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>震傳媒（委山水執行）</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1070</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>li:39.6,su:34.8</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>li:32.0,su:28.0</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://www.zmedia.com.tw/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>nt2026-002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>asia-pacific</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>新台灣國策智庫</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E4" t="n">
         <v>1083</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>phone</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
         <v>2.97</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>li:40.0,su:40.2</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>li:33.0,su:34.0</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="J4" t="n">
         <v>19.8</v>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>http://www.braintrust.tw/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>nt2026-003</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>junews</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>鉅聞天下新聞網（委皮爾森數據）</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1766</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>li:50.85,su:44.06</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>li:54.81,su:33.21</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://www.ftnn.com.tw/</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1403,6 +1505,57 @@
       <c r="K4" t="inlineStr">
         <is>
           <t>https://news.tvbs.com.tw/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>tp2026-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>zmedia</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>震傳媒（委山水執行）</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1074</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>chiang:55.2,shen:27.5</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>chiang:47.0,shen:10.2</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://www.zmedia.com.tw/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: register Era News and add new July 20 Kaohsiung Mayor poll (Lai 36.2% vs Ke 23.6%)
</commit_message>
<xml_diff>
--- a/sheets_import/clearpoll_database.xlsx
+++ b/sheets_import/clearpoll_database.xlsx
@@ -918,7 +918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1281,6 +1281,57 @@
       <c r="K7" t="inlineStr">
         <is>
           <t>https://www.ettoday.net/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>kh2026-005</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>era</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>年代民調</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1068</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>lai:36.2,ke:23.6</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>lai:28.0,ke:20.0</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://news.nexttv.com.tw/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: correct July 20 Kaohsiung Era News poll with exact crosstab data (sample 1071, neutral results Lai 10.6% vs Ke 17.4%)
</commit_message>
<xml_diff>
--- a/sheets_import/clearpoll_database.xlsx
+++ b/sheets_import/clearpoll_database.xlsx
@@ -1306,7 +1306,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1068</v>
+        <v>1071</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>lai:28.0,ke:20.0</t>
+          <t>lai:10.6,ke:17.4</t>
         </is>
       </c>
       <c r="J8" t="n">

</xml_diff>

<commit_message>
feat: add April 13 Formosa and May 12 ETtoday polls to New Taipei City 2026 to increase data completeness
</commit_message>
<xml_diff>
--- a/sheets_import/clearpoll_database.xlsx
+++ b/sheets_import/clearpoll_database.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -533,22 +533,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>nt2026-001b</t>
+          <t>nt2026-001c</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>zmedia</t>
+          <t>formosa</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>震傳媒（委山水執行）</t>
+          <t>美麗島</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -564,46 +564,46 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>li:39.6,su:34.8</t>
+          <t>li:35.5,su:34.5</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>li:32.0,su:28.0</t>
+          <t>li:28.0,su:27.0</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>25.6</v>
+        <v>30</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://www.zmedia.com.tw/</t>
+          <t>https://www.my-formosa.com/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>nt2026-002</t>
+          <t>nt2026-001b</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>asia-pacific</t>
+          <t>zmedia</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>新台灣國策智庫</t>
+          <t>震傳媒（委山水執行）</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1083</v>
+        <v>1070</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -611,73 +611,175 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>2.97</v>
+        <v>3</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>li:40.0,su:40.2</t>
+          <t>li:39.6,su:34.8</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>li:33.0,su:34.0</t>
+          <t>li:32.0,su:28.0</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>19.8</v>
+        <v>25.6</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>http://www.braintrust.tw/</t>
+          <t>https://www.zmedia.com.tw/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>nt2026-001d</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ettoday</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ETtoday</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1142</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>li:42.5,su:41.7</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>li:35.0,su:34.0</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://www.ettoday.net/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>nt2026-002</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>asia-pacific</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>新台灣國策智庫</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1083</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>li:40.0,su:40.2</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>li:33.0,su:34.0</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>http://www.braintrust.tw/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>nt2026-003</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>junews</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>鉅聞天下新聞網（委皮爾森數據）</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E7" t="n">
         <v>1766</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>online</t>
         </is>
       </c>
-      <c r="G5" t="n">
+      <c r="G7" t="n">
         <v>2.3</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>li:50.85,su:44.06</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>li:54.81,su:33.21</t>
         </is>
       </c>
-      <c r="J5" t="n">
+      <c r="J7" t="n">
         <v>5.09</v>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>https://www.ftnn.com.tw/</t>
         </is>

</xml_diff>

<commit_message>
feat: upgrade model with House Effect Calibration, Monte Carlo 95% CIs, Scenario Simulator, Poll Details Modal, and poll expansion
</commit_message>
<xml_diff>
--- a/sheets_import/clearpoll_database.xlsx
+++ b/sheets_import/clearpoll_database.xlsx
@@ -796,7 +796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1006,6 +1006,108 @@
       <c r="K4" t="inlineStr">
         <is>
           <t>https://cnews.com.tw/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>tc2026-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>tvbs</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>TVBS</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1110</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>chiang_k:52.0,ho:31.0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>chiang_k:43.0,ho:25.0</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>17</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://news.tvbs.com.tw/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>tc2026-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>formosa</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>美麗島</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1075</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>chiang_k:49.5,ho:33.5</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>chiang_k:41.0,ho:27.0</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>17</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://www.my-formosa.com/</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1882,6 +1984,108 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>https://news.tvbs.com.tw/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>tn2026-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>formosa</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>美麗島</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1072</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>chen_t:51.5,hsie:32.5</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>chen_t:43.0,hsie:26.0</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>16</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://www.my-formosa.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>tn2026-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>era</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>年代民調</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1060</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>chen_t:48.0,hsie:35.0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>chen_t:39.0,hsie:29.0</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>17</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://www.eranews.com.tw/</t>
         </is>
       </c>
     </row>
@@ -1896,7 +2100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2010,51 +2214,153 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>ty2026-001b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ettoday</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ETtoday</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1080</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>chang:56.5,huang:24.5</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>chang:46.0,huang:20.0</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>19</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://www.ettoday.net/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>ty2026-002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>cnews</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>匯流新聞網</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E4" t="n">
         <v>1050</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>phone</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
         <v>3.02</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>chang:54.0,huang:25.0</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>chang:44.0,huang:21.0</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="J4" t="n">
         <v>21</v>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>https://cnews.com.tw/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ty2026-003</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>era</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>年代民調</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1065</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>chang:52.0,huang:27.0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>chang:42.0,huang:22.0</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>21</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://www.eranews.com.tw/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add 7/23 ZMedia Kaohsiung poll and implement CDPSM dynamic partisan demographics model
</commit_message>
<xml_diff>
--- a/sheets_import/clearpoll_database.xlsx
+++ b/sheets_import/clearpoll_database.xlsx
@@ -1122,7 +1122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1536,6 +1536,53 @@
       <c r="K8" t="inlineStr">
         <is>
           <t>https://www.eranews.com.tw/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>kh2026-006</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>zmedia</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>震傳媒</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1071</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>lai:39.6,ke:31.6</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://www.zmedia.com.tw/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: add newly published TVBS poll for New Taipei Mayor (2026-07-29)
</commit_message>
<xml_diff>
--- a/sheets_import/clearpoll_database.xlsx
+++ b/sheets_import/clearpoll_database.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -782,6 +782,57 @@
       <c r="K7" t="inlineStr">
         <is>
           <t>https://www.ftnn.com.tw/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>nt2026-004</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>tvbs</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>TVBS</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1050</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>li:43.7,su:36.8</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>li:36.0,su:30.0</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://news.tvbs.com.tw/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: update with latest August 2026 polls for Taichung (艾普羅) and Kaohsiung (鉅聞天下)
</commit_message>
<xml_diff>
--- a/sheets_import/clearpoll_database.xlsx
+++ b/sheets_import/clearpoll_database.xlsx
@@ -847,7 +847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1159,6 +1159,57 @@
       <c r="K6" t="inlineStr">
         <is>
           <t>https://www.my-formosa.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>tc2026-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>cnews</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>艾普羅</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1077</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>chiang_k:38.2,ho:24.1</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>chiang_k:32.0,ho:20.0</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://cnews.com.tw/</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1634,6 +1685,57 @@
       <c r="K9" t="inlineStr">
         <is>
           <t>https://www.zmedia.com.tw/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>kh2026-007</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>junews</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>鉅聞天下（委皮爾森執行）</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1608</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>lai:47.78,ke:46.14</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>lai:45.0,ke:43.0</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://www.ftnn.com.tw/</t>
         </is>
       </c>
     </row>

</xml_diff>